<commit_message>
excluye revion de documentos
</commit_message>
<xml_diff>
--- a/UtilesEscolares.xlsx
+++ b/UtilesEscolares.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\ChatBots\LaptopsUtilesEscolares\pc-venta-ia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A72EAAE0-C025-48DB-B16E-E3D5E68598E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2D7A280-0757-4083-A661-CFCEED5F6F08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7EA849BD-3D9F-4698-BFE7-A1933C0DBA1F}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{7EA849BD-3D9F-4698-BFE7-A1933C0DBA1F}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="104">
   <si>
     <t>Producto</t>
   </si>
@@ -62,15 +62,6 @@
     <t>Modelos: Pelota fitbol, atronauta,Spiderman, hello Kitty, Unicornio, Sofía</t>
   </si>
   <si>
-    <t>Mochila escolar 3 en 1</t>
-  </si>
-  <si>
-    <t>MOCHILA COD 63974</t>
-  </si>
-  <si>
-    <t>MOCHILA TOTO DE NIÑA NUEVO LOGO</t>
-  </si>
-  <si>
     <t>Kit MOCHILA TOTO</t>
   </si>
   <si>
@@ -200,9 +191,6 @@
     <t>Goma Blanca Bester Multipropósito 120 g</t>
   </si>
   <si>
-    <t>Tijera Escolar Bester</t>
-  </si>
-  <si>
     <t>Acero inoxidable,Punta redonda</t>
   </si>
   <si>
@@ -264,6 +252,105 @@
   </si>
   <si>
     <t>Fomix  llano</t>
+  </si>
+  <si>
+    <t>MOCHILA COD 65240</t>
+  </si>
+  <si>
+    <t>kit Mochila escolar 3 en 1 con luz</t>
+  </si>
+  <si>
+    <t>MOCHILA TOTO DE NIÑA NUEVO LOGO cod 2610</t>
+  </si>
+  <si>
+    <t>Kit mochila Totto cod 2604</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incluye: Mochila, cartuchera y lonchera </t>
+  </si>
+  <si>
+    <t>Mochila infantil cod 9125 spiderman</t>
+  </si>
+  <si>
+    <t>Rompecabezas 15x15cm 53008</t>
+  </si>
+  <si>
+    <t>9 piezas</t>
+  </si>
+  <si>
+    <t>Rompecabezas didactico 740</t>
+  </si>
+  <si>
+    <t>menores de 3 años</t>
+  </si>
+  <si>
+    <t>Rompecabezas de letras de madera</t>
+  </si>
+  <si>
+    <t>Rompecabezas 3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16x16cm </t>
+  </si>
+  <si>
+    <t>Cuaderno pequeño cuadros espiral  que enamora</t>
+  </si>
+  <si>
+    <t>espiral cuadros</t>
+  </si>
+  <si>
+    <t>Cuaderno universitario cuadros 100 hojas</t>
+  </si>
+  <si>
+    <t>marca zien, 100 h</t>
+  </si>
+  <si>
+    <t>Pinturas x12 pequeñas</t>
+  </si>
+  <si>
+    <t>caja pequeña de 12 pinturas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pinturas x24 mazh premium </t>
+  </si>
+  <si>
+    <t>24 pinturas gruesas 4mm</t>
+  </si>
+  <si>
+    <t>pinturas x12craft premium</t>
+  </si>
+  <si>
+    <t>16 colores con sacapuntas</t>
+  </si>
+  <si>
+    <t>Cuaderno cosido 100 hojas cuadros</t>
+  </si>
+  <si>
+    <t>Papel crepe x10 paquete</t>
+  </si>
+  <si>
+    <t>Rega de goma flexible 30 cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cartulina Iris A4 </t>
+  </si>
+  <si>
+    <t>paquete 10 colores</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tijera Escolar Bester </t>
+  </si>
+  <si>
+    <t>14 cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pinturas x 15 mazh premium </t>
+  </si>
+  <si>
+    <t>15 pinturas 3mm</t>
+  </si>
+  <si>
+    <t>Tijera Escolar Bester punta redonda</t>
   </si>
 </sst>
 </file>
@@ -368,6 +455,25 @@
   <dxfs count="4">
     <dxf>
       <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FFC00000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -423,25 +529,6 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FFC00000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -558,17 +645,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{546F2D59-2300-4F2F-8662-51972628AA21}" name="Tabla1" displayName="Tabla1" ref="A1:C41" totalsRowShown="0" headerRowDxfId="3">
-  <autoFilter ref="A1:C41" xr:uid="{546F2D59-2300-4F2F-8662-51972628AA21}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{546F2D59-2300-4F2F-8662-51972628AA21}" name="Tabla1" displayName="Tabla1" ref="A1:C1048576" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:C1048576" xr:uid="{546F2D59-2300-4F2F-8662-51972628AA21}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C41">
     <sortCondition ref="A1:A41"/>
   </sortState>
   <tableColumns count="3">
-    <tableColumn id="2" xr3:uid="{07407FDA-9294-4728-8AAE-A67E755034AC}" name="Producto" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{B30E59F2-CA4E-4991-9A00-04C98A38D233}" name="Descripcion" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{4490A5B2-BE38-49F1-8AA2-1F7E3D2EF485}" name="Precio de venta al publico " dataDxfId="0">
-      <calculatedColumnFormula>#REF!+(#REF!*0.6)</calculatedColumnFormula>
-    </tableColumn>
+    <tableColumn id="2" xr3:uid="{07407FDA-9294-4728-8AAE-A67E755034AC}" name="Producto" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{B30E59F2-CA4E-4991-9A00-04C98A38D233}" name="Descripcion" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{4490A5B2-BE38-49F1-8AA2-1F7E3D2EF485}" name="Precio de venta al publico " dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -891,7 +976,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D24BF651-7A97-4644-9956-DED6372BC8A8}">
-  <dimension ref="A1:C119"/>
+  <dimension ref="A1:C136"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="43.26953125" style="8" customWidth="1"/>
@@ -912,10 +997,10 @@
     </row>
     <row r="2" spans="1:3" s="2" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="7" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C2" s="10">
         <v>1.58</v>
@@ -923,10 +1008,10 @@
     </row>
     <row r="3" spans="1:3" s="2" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C3" s="10">
         <v>0.4</v>
@@ -934,10 +1019,10 @@
     </row>
     <row r="4" spans="1:3" s="2" customFormat="1" ht="25" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C4" s="10">
         <v>14.38</v>
@@ -945,10 +1030,10 @@
     </row>
     <row r="5" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C5" s="10">
         <v>3.6</v>
@@ -956,10 +1041,10 @@
     </row>
     <row r="6" spans="1:3" s="2" customFormat="1" ht="25" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C6" s="10">
         <v>3.6</v>
@@ -967,10 +1052,10 @@
     </row>
     <row r="7" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C7" s="10">
         <v>3.6</v>
@@ -989,10 +1074,10 @@
     </row>
     <row r="9" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A9" s="7" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C9" s="10">
         <v>1.28</v>
@@ -1000,7 +1085,7 @@
     </row>
     <row r="10" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="7" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B10" s="7"/>
       <c r="C10" s="10">
@@ -1009,10 +1094,10 @@
     </row>
     <row r="11" spans="1:3" s="2" customFormat="1" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A11" s="7" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C11" s="10">
         <v>1.58</v>
@@ -1020,10 +1105,10 @@
     </row>
     <row r="12" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A12" s="6" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C12" s="10">
         <v>0.77</v>
@@ -1031,7 +1116,7 @@
     </row>
     <row r="13" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A13" s="7" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="10">
@@ -1040,10 +1125,10 @@
     </row>
     <row r="14" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C14" s="10">
         <v>4.78</v>
@@ -1051,10 +1136,10 @@
     </row>
     <row r="15" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C15" s="10">
         <v>1.58</v>
@@ -1062,10 +1147,10 @@
     </row>
     <row r="16" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C16" s="10">
         <v>2.8</v>
@@ -1073,10 +1158,10 @@
     </row>
     <row r="17" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A17" s="6" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C17" s="10">
         <v>1.2</v>
@@ -1084,10 +1169,10 @@
     </row>
     <row r="18" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A18" s="7" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C18" s="10">
         <v>2.3199999999999998</v>
@@ -1095,10 +1180,10 @@
     </row>
     <row r="19" spans="1:3" s="2" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="7" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C19" s="10">
         <v>0.64</v>
@@ -1106,10 +1191,10 @@
     </row>
     <row r="20" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" s="7" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C20" s="10">
         <v>0.56000000000000005</v>
@@ -1117,10 +1202,10 @@
     </row>
     <row r="21" spans="1:3" s="2" customFormat="1" ht="25" x14ac:dyDescent="0.35">
       <c r="A21" s="7" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C21" s="10">
         <v>0.88</v>
@@ -1128,10 +1213,10 @@
     </row>
     <row r="22" spans="1:3" s="2" customFormat="1" ht="25" x14ac:dyDescent="0.35">
       <c r="A22" s="7" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C22" s="10">
         <v>1.36</v>
@@ -1139,10 +1224,10 @@
     </row>
     <row r="23" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A23" s="6" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C23" s="10">
         <v>25.58</v>
@@ -1150,10 +1235,10 @@
     </row>
     <row r="24" spans="1:3" s="2" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="7" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C24" s="10">
         <v>0.48</v>
@@ -1161,10 +1246,10 @@
     </row>
     <row r="25" spans="1:3" s="2" customFormat="1" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="7" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C25" s="10">
         <v>0.4</v>
@@ -1172,10 +1257,10 @@
     </row>
     <row r="26" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A26" s="7" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C26" s="10">
         <v>1.36</v>
@@ -1183,10 +1268,10 @@
     </row>
     <row r="27" spans="1:3" s="2" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="7" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C27" s="10">
         <v>1.36</v>
@@ -1194,10 +1279,10 @@
     </row>
     <row r="28" spans="1:3" s="2" customFormat="1" ht="25" x14ac:dyDescent="0.35">
       <c r="A28" s="7" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C28" s="10">
         <v>0.96</v>
@@ -1216,10 +1301,10 @@
     </row>
     <row r="30" spans="1:3" s="2" customFormat="1" ht="25" x14ac:dyDescent="0.35">
       <c r="A30" s="7" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C30" s="10">
         <v>0.88</v>
@@ -1227,10 +1312,10 @@
     </row>
     <row r="31" spans="1:3" s="2" customFormat="1" ht="25" x14ac:dyDescent="0.35">
       <c r="A31" s="7" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C31" s="10">
         <v>0.88</v>
@@ -1238,19 +1323,19 @@
     </row>
     <row r="32" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A32" s="7" t="s">
-        <v>8</v>
+        <v>71</v>
       </c>
       <c r="B32" s="7"/>
       <c r="C32" s="10">
-        <v>8.8000000000000007</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="33" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A33" s="7" t="s">
-        <v>7</v>
+        <v>72</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C33" s="10">
         <v>15.98</v>
@@ -1258,7 +1343,7 @@
     </row>
     <row r="34" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A34" s="7" t="s">
-        <v>9</v>
+        <v>73</v>
       </c>
       <c r="B34" s="7"/>
       <c r="C34" s="10">
@@ -1267,10 +1352,10 @@
     </row>
     <row r="35" spans="1:3" s="2" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="6" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C35" s="10">
         <v>7.2</v>
@@ -1278,10 +1363,10 @@
     </row>
     <row r="36" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A36" s="7" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C36" s="10">
         <v>0.45</v>
@@ -1289,10 +1374,10 @@
     </row>
     <row r="37" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A37" s="6" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C37" s="10">
         <v>1.84</v>
@@ -1300,10 +1385,10 @@
     </row>
     <row r="38" spans="1:3" s="2" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="7" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C38" s="10">
         <v>1.36</v>
@@ -1311,10 +1396,10 @@
     </row>
     <row r="39" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A39" s="7" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C39" s="10">
         <v>2.96</v>
@@ -1322,7 +1407,7 @@
     </row>
     <row r="40" spans="1:3" s="2" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="7" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B40" s="4"/>
       <c r="C40" s="10">
@@ -1331,99 +1416,191 @@
     </row>
     <row r="41" spans="1:3" s="2" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="B41" s="4" t="s">
-        <v>54</v>
+        <v>74</v>
+      </c>
+      <c r="B41" s="7" t="s">
+        <v>75</v>
       </c>
       <c r="C41" s="10">
+        <v>28.99</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="B42" s="7"/>
+      <c r="C42" s="10">
+        <v>9.25</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A43" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C43" s="10">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B44" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="C44" s="10">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="B45" s="7"/>
+      <c r="C45" s="10">
+        <v>4.25</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B46" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C46" s="10">
+        <v>2.2000000000000002</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="B47" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="C47" s="10">
+        <v>1.58</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A48" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="B48" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="C48" s="10">
+        <v>1.76</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A49" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B49" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="C49" s="10">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A50" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="B50" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="C50" s="10">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A51" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B51" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="C51" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A52" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="B52" s="7"/>
+      <c r="C52" s="10">
+        <v>1.76</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A53" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="B53" s="7"/>
+      <c r="C53" s="10">
+        <v>3.18</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A54" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B54" s="7"/>
+      <c r="C54" s="10">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A55" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="B55" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="C55" s="10">
+        <v>1.04</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A56" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="B56" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C56" s="10">
+        <v>3.18</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A57" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="B57" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="C57" s="10">
+        <v>2.2000000000000002</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A58" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C58" s="10">
         <v>1.2</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="6"/>
-      <c r="B42" s="4"/>
-      <c r="C42" s="5"/>
-    </row>
-    <row r="43" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="6"/>
-      <c r="B43" s="4"/>
-      <c r="C43" s="5"/>
-    </row>
-    <row r="44" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="6"/>
-      <c r="B44" s="4"/>
-      <c r="C44" s="5"/>
-    </row>
-    <row r="45" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="6"/>
-      <c r="B45" s="4"/>
-      <c r="C45" s="5"/>
-    </row>
-    <row r="46" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="6"/>
-      <c r="B46" s="4"/>
-      <c r="C46" s="5"/>
-    </row>
-    <row r="47" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="6"/>
-      <c r="B47" s="4"/>
-      <c r="C47" s="5"/>
-    </row>
-    <row r="48" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="6"/>
-      <c r="B48" s="4"/>
-      <c r="C48" s="5"/>
-    </row>
-    <row r="49" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="6"/>
-      <c r="B49" s="4"/>
-      <c r="C49" s="5"/>
-    </row>
-    <row r="50" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="6"/>
-      <c r="B50" s="4"/>
-      <c r="C50" s="5"/>
-    </row>
-    <row r="51" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="6"/>
-      <c r="B51" s="4"/>
-      <c r="C51" s="5"/>
-    </row>
-    <row r="52" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="6"/>
-      <c r="B52" s="4"/>
-      <c r="C52" s="5"/>
-    </row>
-    <row r="53" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="6"/>
-      <c r="B53" s="4"/>
-      <c r="C53" s="5"/>
-    </row>
-    <row r="54" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="6"/>
-      <c r="B54" s="4"/>
-      <c r="C54" s="5"/>
-    </row>
-    <row r="55" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="6"/>
-      <c r="B55" s="4"/>
-      <c r="C55" s="5"/>
-    </row>
-    <row r="56" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="6"/>
-      <c r="B56" s="4"/>
-      <c r="C56" s="5"/>
-    </row>
-    <row r="57" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A57" s="6"/>
-      <c r="B57" s="4"/>
-      <c r="C57" s="5"/>
-    </row>
-    <row r="58" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A58" s="6"/>
-      <c r="B58" s="4"/>
-      <c r="C58" s="5"/>
     </row>
     <row r="59" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A59" s="6"/>
@@ -1729,6 +1906,74 @@
       <c r="A119" s="6"/>
       <c r="B119" s="4"/>
       <c r="C119" s="5"/>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A120" s="6"/>
+      <c r="B120" s="4"/>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A121" s="6"/>
+      <c r="B121" s="4"/>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A122" s="6"/>
+      <c r="B122" s="4"/>
+    </row>
+    <row r="123" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A123" s="6"/>
+      <c r="B123" s="4"/>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A124" s="6"/>
+      <c r="B124" s="4"/>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A125" s="6"/>
+      <c r="B125" s="4"/>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A126" s="6"/>
+      <c r="B126" s="4"/>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A127" s="6"/>
+      <c r="B127" s="4"/>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A128" s="6"/>
+      <c r="B128" s="4"/>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A129" s="6"/>
+      <c r="B129" s="4"/>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A130" s="6"/>
+      <c r="B130" s="4"/>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A131" s="6"/>
+      <c r="B131" s="4"/>
+    </row>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A132" s="6"/>
+      <c r="B132" s="4"/>
+    </row>
+    <row r="133" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A133" s="6"/>
+      <c r="B133" s="4"/>
+    </row>
+    <row r="134" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A134" s="6"/>
+      <c r="B134" s="4"/>
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A135" s="6"/>
+      <c r="B135" s="4"/>
+    </row>
+    <row r="136" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A136" s="6"/>
+      <c r="B136" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Fotos de productos: carpeta imagenes/ (numeradas por producto) y envio via IA (enviar_foto); catalogo actualizado a 59 productos
</commit_message>
<xml_diff>
--- a/UtilesEscolares.xlsx
+++ b/UtilesEscolares.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\ChatBots\LaptopsUtilesEscolares\pc-venta-ia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31B613AC-EB4E-4CB4-9134-D97766264648}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C960F26-DDF5-43EA-B117-697E5D9E6C87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7EA849BD-3D9F-4698-BFE7-A1933C0DBA1F}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="63">
   <si>
     <t>Producto</t>
   </si>
@@ -222,13 +222,19 @@
   </si>
   <si>
     <t>Esfero rojo triangular bester  punta fina de 0.7 mm</t>
+  </si>
+  <si>
+    <t>Mochila cod 65531</t>
+  </si>
+  <si>
+    <t>Mochila cod 65136</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -269,6 +275,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -290,7 +302,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -316,6 +328,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -338,7 +351,8 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -357,8 +371,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -465,13 +478,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>55</xdr:row>
+      <xdr:row>56</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>56</xdr:row>
+      <xdr:row>57</xdr:row>
       <xdr:rowOff>120650</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -515,13 +528,13 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{546F2D59-2300-4F2F-8662-51972628AA21}" name="Tabla1" displayName="Tabla1" ref="A1:C1048576" totalsRowShown="0" headerRowDxfId="3">
   <autoFilter ref="A1:C1048576" xr:uid="{546F2D59-2300-4F2F-8662-51972628AA21}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C137">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C119">
     <sortCondition ref="B1:B1048576"/>
   </sortState>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{B34F359A-0389-42A2-90C4-2EB25D08220D}" name="Número de producto" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{07407FDA-9294-4728-8AAE-A67E755034AC}" name="Producto" dataDxfId="0"/>
-    <tableColumn id="5" xr3:uid="{4490A5B2-BE38-49F1-8AA2-1F7E3D2EF485}" name="Precio de venta al publico " dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{07407FDA-9294-4728-8AAE-A67E755034AC}" name="Producto" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{4490A5B2-BE38-49F1-8AA2-1F7E3D2EF485}" name="Precio de venta al publico " dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -870,10 +883,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="C2" s="6">
-        <v>0.45</v>
+        <v>1.58</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="2" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -882,10 +895,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C3" s="6">
-        <v>1.58</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -894,10 +907,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C4" s="6">
-        <v>0.4</v>
+        <v>13.38</v>
       </c>
     </row>
     <row r="5" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -906,10 +919,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C5" s="6">
-        <v>13.38</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="6" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -918,10 +931,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C6" s="6">
-        <v>3.6</v>
+        <v>1.04</v>
       </c>
     </row>
     <row r="7" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -930,10 +943,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C7" s="6">
-        <v>1.04</v>
+        <v>1.28</v>
       </c>
     </row>
     <row r="8" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -942,10 +955,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C8" s="6">
-        <v>1.28</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="9" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -954,10 +967,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C9" s="6">
-        <v>0.88</v>
+        <v>1.58</v>
       </c>
     </row>
     <row r="10" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -966,10 +979,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C10" s="6">
-        <v>1.58</v>
+        <v>0.77</v>
       </c>
     </row>
     <row r="11" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -978,10 +991,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="C11" s="6">
-        <v>0.77</v>
+        <v>1.76</v>
       </c>
     </row>
     <row r="12" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -990,10 +1003,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C12" s="6">
-        <v>1.76</v>
+        <v>1.58</v>
       </c>
     </row>
     <row r="13" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1002,10 +1015,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C13" s="6">
-        <v>1.58</v>
+        <v>1.76</v>
       </c>
     </row>
     <row r="14" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1014,10 +1027,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="C14" s="6">
-        <v>1.76</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1026,10 +1039,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C15" s="6">
-        <v>2</v>
+        <v>4.78</v>
       </c>
     </row>
     <row r="16" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1038,10 +1051,10 @@
         <v>15</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C16" s="6">
-        <v>4.78</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="17" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1050,10 +1063,10 @@
         <v>16</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C17" s="6">
-        <v>0.45</v>
+        <v>26</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1062,10 +1075,10 @@
         <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>13</v>
+        <v>60</v>
+      </c>
+      <c r="C18" s="6">
+        <v>0.45</v>
       </c>
     </row>
     <row r="19" spans="1:3" s="2" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1308,16 +1321,16 @@
         <v>13.5</v>
       </c>
     </row>
-    <row r="39" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:3" s="2" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="5">
         <f>ROW()-1</f>
         <v>38</v>
       </c>
-      <c r="B39" s="4" t="s">
-        <v>2</v>
+      <c r="B39" s="9" t="s">
+        <v>61</v>
       </c>
       <c r="C39" s="6">
-        <v>9.25</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="40" spans="1:3" s="2" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1326,10 +1339,10 @@
         <v>39</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>47</v>
+        <v>2</v>
       </c>
       <c r="C40" s="6">
-        <v>15.98</v>
+        <v>9.25</v>
       </c>
     </row>
     <row r="41" spans="1:3" s="2" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1338,10 +1351,10 @@
         <v>40</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>7</v>
+        <v>47</v>
       </c>
       <c r="C41" s="6">
-        <v>3.18</v>
+        <v>15.98</v>
       </c>
     </row>
     <row r="42" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1350,10 +1363,10 @@
         <v>41</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>48</v>
+        <v>7</v>
       </c>
       <c r="C42" s="6">
-        <v>7.2</v>
+        <v>3.18</v>
       </c>
     </row>
     <row r="43" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1362,10 +1375,10 @@
         <v>42</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C43" s="6">
-        <v>3.6</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="44" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1374,10 +1387,10 @@
         <v>43</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C44" s="6">
-        <v>2.2000000000000002</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="45" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1386,10 +1399,10 @@
         <v>44</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C45" s="6">
-        <v>2</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="46" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1398,10 +1411,10 @@
         <v>45</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>5</v>
+        <v>51</v>
       </c>
       <c r="C46" s="6">
-        <v>0.6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1410,10 +1423,10 @@
         <v>46</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C47" s="6">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="48" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1422,10 +1435,10 @@
         <v>47</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>52</v>
+        <v>8</v>
       </c>
       <c r="C48" s="6">
-        <v>0.45</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="49" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1434,10 +1447,10 @@
         <v>48</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>11</v>
+        <v>52</v>
       </c>
       <c r="C49" s="6">
-        <v>0.75</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="50" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1446,10 +1459,10 @@
         <v>49</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>53</v>
+        <v>11</v>
       </c>
       <c r="C50" s="6">
-        <v>2.2000000000000002</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="51" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1458,10 +1471,10 @@
         <v>50</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>4</v>
+        <v>53</v>
       </c>
       <c r="C51" s="6">
-        <v>4.25</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="52" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1470,10 +1483,10 @@
         <v>51</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C52" s="6">
-        <v>5.5</v>
+        <v>4.25</v>
       </c>
     </row>
     <row r="53" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1482,10 +1495,10 @@
         <v>52</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>54</v>
+        <v>3</v>
       </c>
       <c r="C53" s="6">
-        <v>1.84</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="54" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1494,10 +1507,10 @@
         <v>53</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C54" s="6">
-        <v>1.36</v>
+        <v>1.84</v>
       </c>
     </row>
     <row r="55" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1506,10 +1519,10 @@
         <v>54</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C55" s="6">
-        <v>2.96</v>
+        <v>1.36</v>
       </c>
     </row>
     <row r="56" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1518,7 +1531,7 @@
         <v>55</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C56" s="6">
         <v>2.96</v>
@@ -1530,10 +1543,10 @@
         <v>56</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C57" s="6">
-        <v>3.18</v>
+        <v>2.96</v>
       </c>
     </row>
     <row r="58" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1542,21 +1555,35 @@
         <v>57</v>
       </c>
       <c r="B58" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C58" s="6">
+        <v>3.18</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" s="2" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A59" s="5">
+        <f>ROW()-1</f>
+        <v>58</v>
+      </c>
+      <c r="B59" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="C58" s="6">
+      <c r="C59" s="6">
         <v>1.2</v>
       </c>
     </row>
-    <row r="59" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A59" s="5"/>
-      <c r="B59" s="4"/>
-      <c r="C59" s="3"/>
-    </row>
     <row r="60" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A60" s="5"/>
-      <c r="B60" s="4"/>
-      <c r="C60" s="3"/>
+      <c r="A60" s="5">
+        <f>ROW()-1</f>
+        <v>59</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C60" s="6">
+        <v>16</v>
+      </c>
     </row>
     <row r="61" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A61" s="5"/>

</xml_diff>

<commit_message>
Comprobante verificado con IA (monto >= 50% y titular Evelyn Zambrano) al llegar la imagen; tras la confirmacion del pedido no se envian mas mensajes
</commit_message>
<xml_diff>
--- a/UtilesEscolares.xlsx
+++ b/UtilesEscolares.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\ChatBots\LaptopsUtilesEscolares\pc-venta-ia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C960F26-DDF5-43EA-B117-697E5D9E6C87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CBCC33A-9EC4-4911-BAA6-2EE0BDE82005}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7EA849BD-3D9F-4698-BFE7-A1933C0DBA1F}"/>
   </bookViews>
@@ -879,7 +879,7 @@
     </row>
     <row r="2" spans="1:3" s="2" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" ref="A2:A33" si="0">ROW()-1</f>
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
@@ -891,7 +891,7 @@
     </row>
     <row r="3" spans="1:3" s="2" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
@@ -903,7 +903,7 @@
     </row>
     <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
@@ -915,7 +915,7 @@
     </row>
     <row r="5" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
@@ -927,7 +927,7 @@
     </row>
     <row r="6" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
@@ -939,7 +939,7 @@
     </row>
     <row r="7" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
@@ -951,7 +951,7 @@
     </row>
     <row r="8" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
@@ -963,7 +963,7 @@
     </row>
     <row r="9" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
@@ -975,7 +975,7 @@
     </row>
     <row r="10" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
@@ -987,7 +987,7 @@
     </row>
     <row r="11" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
@@ -999,7 +999,7 @@
     </row>
     <row r="12" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
@@ -1011,7 +1011,7 @@
     </row>
     <row r="13" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
@@ -1023,7 +1023,7 @@
     </row>
     <row r="14" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
@@ -1035,7 +1035,7 @@
     </row>
     <row r="15" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
@@ -1047,7 +1047,7 @@
     </row>
     <row r="16" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="B16" s="4" t="s">
@@ -1059,7 +1059,7 @@
     </row>
     <row r="17" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="B17" s="4" t="s">
@@ -1071,7 +1071,7 @@
     </row>
     <row r="18" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
@@ -1083,7 +1083,7 @@
     </row>
     <row r="19" spans="1:3" s="2" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="B19" s="4" t="s">
@@ -1095,7 +1095,7 @@
     </row>
     <row r="20" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="B20" s="4" t="s">
@@ -1107,7 +1107,7 @@
     </row>
     <row r="21" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="B21" s="4" t="s">
@@ -1119,7 +1119,7 @@
     </row>
     <row r="22" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="B22" s="4" t="s">
@@ -1131,7 +1131,7 @@
     </row>
     <row r="23" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="B23" s="4" t="s">
@@ -1143,7 +1143,7 @@
     </row>
     <row r="24" spans="1:3" s="2" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="B24" s="4" t="s">
@@ -1155,7 +1155,7 @@
     </row>
     <row r="25" spans="1:3" s="2" customFormat="1" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="B25" s="4" t="s">
@@ -1167,7 +1167,7 @@
     </row>
     <row r="26" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A26" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>25</v>
       </c>
       <c r="B26" s="4" t="s">
@@ -1179,7 +1179,7 @@
     </row>
     <row r="27" spans="1:3" s="2" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>26</v>
       </c>
       <c r="B27" s="4" t="s">
@@ -1191,7 +1191,7 @@
     </row>
     <row r="28" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>27</v>
       </c>
       <c r="B28" s="4" t="s">
@@ -1203,7 +1203,7 @@
     </row>
     <row r="29" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A29" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>28</v>
       </c>
       <c r="B29" s="4" t="s">
@@ -1215,7 +1215,7 @@
     </row>
     <row r="30" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A30" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>29</v>
       </c>
       <c r="B30" s="4" t="s">
@@ -1227,7 +1227,7 @@
     </row>
     <row r="31" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A31" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="B31" s="4" t="s">
@@ -1239,7 +1239,7 @@
     </row>
     <row r="32" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>31</v>
       </c>
       <c r="B32" s="4" t="s">
@@ -1251,7 +1251,7 @@
     </row>
     <row r="33" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A33" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="B33" s="4" t="s">
@@ -1263,7 +1263,7 @@
     </row>
     <row r="34" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" ref="A34:A60" si="1">ROW()-1</f>
         <v>33</v>
       </c>
       <c r="B34" s="4" t="s">
@@ -1275,7 +1275,7 @@
     </row>
     <row r="35" spans="1:3" s="2" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="1"/>
         <v>34</v>
       </c>
       <c r="B35" s="4" t="s">
@@ -1287,7 +1287,7 @@
     </row>
     <row r="36" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A36" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="1"/>
         <v>35</v>
       </c>
       <c r="B36" s="4" t="s">
@@ -1299,7 +1299,7 @@
     </row>
     <row r="37" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A37" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="1"/>
         <v>36</v>
       </c>
       <c r="B37" s="4" t="s">
@@ -1311,7 +1311,7 @@
     </row>
     <row r="38" spans="1:3" s="2" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="1"/>
         <v>37</v>
       </c>
       <c r="B38" s="4" t="s">
@@ -1323,7 +1323,7 @@
     </row>
     <row r="39" spans="1:3" s="2" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="1"/>
         <v>38</v>
       </c>
       <c r="B39" s="9" t="s">
@@ -1335,7 +1335,7 @@
     </row>
     <row r="40" spans="1:3" s="2" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="1"/>
         <v>39</v>
       </c>
       <c r="B40" s="4" t="s">
@@ -1347,7 +1347,7 @@
     </row>
     <row r="41" spans="1:3" s="2" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="1"/>
         <v>40</v>
       </c>
       <c r="B41" s="4" t="s">
@@ -1359,7 +1359,7 @@
     </row>
     <row r="42" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A42" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="1"/>
         <v>41</v>
       </c>
       <c r="B42" s="4" t="s">
@@ -1371,7 +1371,7 @@
     </row>
     <row r="43" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A43" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="1"/>
         <v>42</v>
       </c>
       <c r="B43" s="4" t="s">
@@ -1383,7 +1383,7 @@
     </row>
     <row r="44" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A44" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="1"/>
         <v>43</v>
       </c>
       <c r="B44" s="4" t="s">
@@ -1395,7 +1395,7 @@
     </row>
     <row r="45" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A45" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="1"/>
         <v>44</v>
       </c>
       <c r="B45" s="4" t="s">
@@ -1407,7 +1407,7 @@
     </row>
     <row r="46" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A46" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="1"/>
         <v>45</v>
       </c>
       <c r="B46" s="4" t="s">
@@ -1419,7 +1419,7 @@
     </row>
     <row r="47" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A47" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="1"/>
         <v>46</v>
       </c>
       <c r="B47" s="4" t="s">
@@ -1431,7 +1431,7 @@
     </row>
     <row r="48" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A48" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="1"/>
         <v>47</v>
       </c>
       <c r="B48" s="4" t="s">
@@ -1443,7 +1443,7 @@
     </row>
     <row r="49" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A49" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="1"/>
         <v>48</v>
       </c>
       <c r="B49" s="4" t="s">
@@ -1455,7 +1455,7 @@
     </row>
     <row r="50" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A50" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="1"/>
         <v>49</v>
       </c>
       <c r="B50" s="4" t="s">
@@ -1467,7 +1467,7 @@
     </row>
     <row r="51" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A51" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="1"/>
         <v>50</v>
       </c>
       <c r="B51" s="4" t="s">
@@ -1479,7 +1479,7 @@
     </row>
     <row r="52" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A52" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="1"/>
         <v>51</v>
       </c>
       <c r="B52" s="4" t="s">
@@ -1491,7 +1491,7 @@
     </row>
     <row r="53" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A53" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="1"/>
         <v>52</v>
       </c>
       <c r="B53" s="4" t="s">
@@ -1503,7 +1503,7 @@
     </row>
     <row r="54" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A54" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="1"/>
         <v>53</v>
       </c>
       <c r="B54" s="4" t="s">
@@ -1515,7 +1515,7 @@
     </row>
     <row r="55" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A55" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="1"/>
         <v>54</v>
       </c>
       <c r="B55" s="4" t="s">
@@ -1527,7 +1527,7 @@
     </row>
     <row r="56" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A56" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="1"/>
         <v>55</v>
       </c>
       <c r="B56" s="4" t="s">
@@ -1539,7 +1539,7 @@
     </row>
     <row r="57" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A57" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="1"/>
         <v>56</v>
       </c>
       <c r="B57" s="4" t="s">
@@ -1551,7 +1551,7 @@
     </row>
     <row r="58" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A58" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="1"/>
         <v>57</v>
       </c>
       <c r="B58" s="4" t="s">
@@ -1563,7 +1563,7 @@
     </row>
     <row r="59" spans="1:3" s="2" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="1"/>
         <v>58</v>
       </c>
       <c r="B59" s="4" t="s">
@@ -1575,7 +1575,7 @@
     </row>
     <row r="60" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A60" s="5">
-        <f>ROW()-1</f>
+        <f t="shared" si="1"/>
         <v>59</v>
       </c>
       <c r="B60" s="4" t="s">

</xml_diff>